<commit_message>
added agent for button flow
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -29,83 +29,99 @@
     <t>TC001</t>
   </si>
   <si>
-    <t>User starts journey by clicking on "Unlock your saved Payment Options" while logged out on Payu Checkout.</t>
+    <t>User starts journey by clicking on "Unlock your saved Payment Options" when logged out on Payu Checkout.</t>
   </si>
   <si>
     <t>1. Click on "Unlock your saved Payment Options" button.
 2. Enter OTP for vault login.</t>
   </si>
   <si>
-    <t>Pay with Rewards should be shown under preferred payment options with the maximum highest points as sub-text if the user is eligible. If not eligible, Pay with Rewards should not be displayed.</t>
+    <t>Pay with Rewards should be shown under preferred payment options with maximum highest points displayed as sub-text if eligible. If not eligible, Pay with Rewards should not be shown.</t>
   </si>
   <si>
     <t>TC002</t>
   </si>
   <si>
-    <t>User interacts with the expanded accordion after clicking on it.</t>
-  </si>
-  <si>
-    <t>1. Click on the accordion to expand it.
-2. Check if TWID logo is shown on the extreme left.
-3. Click on the cross icon beside TWID logo to close the accordion.
-4. Verify the presence of oval-shaped Earn and Burn buttons.
-5. Check the color of the button based on the merchant flow.</t>
-  </si>
-  <si>
-    <t>TWID logo, cross icon, oval-shaped buttons, and correct button color should be displayed as per the merchant flow.</t>
+    <t>User interacts with the expanded accordion after clicking on "Unlock your saved Payment Options".</t>
+  </si>
+  <si>
+    <t>1. Click on the accordion to expand.
+2. Check for TWID logo and cross icon on the left side.
+3. Verify the presence of earn and burn buttons.
+4. Give consent by checking the checkbox.
+5. Click on the consent checkbox.
+6. Verify the appearance of consent text and rectangular CTAs.</t>
+  </si>
+  <si>
+    <t>Accordion expands showing TWID logo, earn and burn buttons, consent checkbox, and rectangular CTAs as described.</t>
   </si>
   <si>
     <t>TC003</t>
   </si>
   <si>
-    <t>User interacts with the consent checkbox and CTAs.</t>
-  </si>
-  <si>
-    <t>1. Check the color of the consent checkbox.
-2. Read and verify the text of the consent.
-3. Click on the "Change Merchant Name: Coins" CTA and observe the redirection.
-4. Click on the "Pay Rs" CTA and check the loading page.</t>
-  </si>
-  <si>
-    <t>Consent checkbox should be black if given, correct text should be displayed, and CTAs should function as expected.</t>
+    <t>User clicks on "Change Merchant Name</t>
+  </si>
+  <si>
+    <t>1. Click on "Change Merchant Name: Coins" button.
+2. Verify navigation to L2 Page of Rewards.
+3. Check for the presence of a chip with text "Showing Pay with Rewards" and a cross icon.</t>
+  </si>
+  <si>
+    <t>User should be redirected to the L2 Page of Rewards with the expected elements displayed.</t>
   </si>
   <si>
     <t>TC004</t>
   </si>
   <si>
-    <t>User starts journey by clicking on "Pay with Rewards" under the saved Payment Options.</t>
+    <t>User clicks on "Pay Rs" button after selecting a payment method.</t>
+  </si>
+  <si>
+    <t>1. Select a payment method.
+2. Click on "Pay Rs" button.
+3. Verify the appearance of the loading page with Payu Logo.</t>
+  </si>
+  <si>
+    <t>User should be directed to the payment options page with the selected payment method displayed.</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>User starts the journey by clicking on "Pay with Rewards" under the saved Payment Options.</t>
   </si>
   <si>
     <t>1. Click on "Pay with Rewards" under the saved Payment Options.
-2. Enter OTP for vault login.</t>
-  </si>
-  <si>
-    <t>User should land on the L1 page with Pay with Rewards shown under preferred payment options if eligible. Proper messages should be displayed for different eligibility scenarios.</t>
-  </si>
-  <si>
-    <t>TC005</t>
-  </si>
-  <si>
-    <t>User starts journey by clicking on "Pay by Rewards" under the Other Payment Options.</t>
+2. Enter OTP for vault login if required.</t>
+  </si>
+  <si>
+    <t>User should be directed to the L1 page with Pay with Rewards shown under preferred payment options if eligible.</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>User interacts with the L2 Page of Rewards after clicking on "Pay with Rewards" under the saved Payment Options.</t>
+  </si>
+  <si>
+    <t>1. Check for the filtered list on the L2 Page of Rewards.
+2. Verify the display of Pay with Rewards under preferred payment options if eligible.
+3. Check for error messages if not eligible for TWID or other rewards.</t>
+  </si>
+  <si>
+    <t>Correct list and messages should be displayed based on user eligibility.</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>User starts the journey by clicking on "Pay by Rewards" under the Other Payment Options.</t>
   </si>
   <si>
     <t>1. Click on "Pay by Rewards" under the Other Payment Options.
-2. Enter OTP for vault login.</t>
-  </si>
-  <si>
-    <t>User should land on the L2 page with the entire list of rewards shown.</t>
-  </si>
-  <si>
-    <t>TC006</t>
-  </si>
-  <si>
-    <t>User is logged in on Payu Checkout via a previous session/cookie.</t>
-  </si>
-  <si>
-    <t>1. Check if Pay with Rewards is shown under preferred payment options.</t>
-  </si>
-  <si>
-    <t>Pay with Rewards should be displayed with the maximum highest points as sub-text if the user is eligible.</t>
+2. Enter OTP for vault login if required.</t>
+  </si>
+  <si>
+    <t>User should be directed to the L2 page with the entire list of rewards displayed.</t>
   </si>
 </sst>
 </file>
@@ -150,105 +166,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>11</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>15</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" t="s" s="0">
         <v>19</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
+      <c r="A6" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" t="s" s="0">
         <v>23</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s">
+      <c r="A7" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" t="s" s="0">
         <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>